<commit_message>
✨ feat(iol_power_calculator): IOL 計算処理を Excel 対応に更新
</commit_message>
<xml_diff>
--- a/IOLCalcdata.xlsx
+++ b/IOLCalcdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yokam\PycharmProjects\BarrettAutomate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A40343D-9A75-431C-8363-F6773C577E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ADA0CC-545E-4490-91D3-7A8DF1E16560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4620" yWindow="0" windowWidth="17196" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,10 +54,6 @@
     <t>ld</t>
   </si>
   <si>
-    <t>Hoffer PACD</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>eye</t>
   </si>
   <si>
@@ -104,6 +100,10 @@
   </si>
   <si>
     <t>Haisis_SE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Hoffer_pACD</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -542,43 +542,43 @@
         <v>4</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" s="8" t="s">
+      <c r="L1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -592,7 +592,7 @@
         <v>105737</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" s="7">
         <v>23.33</v>
@@ -610,10 +610,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="10">
-        <v>1.88</v>
+        <v>5.37</v>
       </c>
       <c r="K2" s="10">
-        <v>0.9</v>
+        <v>1.9</v>
       </c>
       <c r="L2" s="10">
         <v>0.4</v>

</xml_diff>

<commit_message>
🐛 fix(iol_power_calculator): HofferQ_SE/Haigis_SE 列名のタイポを修正
</commit_message>
<xml_diff>
--- a/IOLCalcdata.xlsx
+++ b/IOLCalcdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yokam\PycharmProjects\BarrettAutomate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ADA0CC-545E-4490-91D3-7A8DF1E16560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92CE348-AD2D-4BCA-86E0-1FEC4E7E9320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4620" yWindow="0" windowWidth="17196" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="696" windowWidth="17196" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="36" r:id="rId1"/>
@@ -99,12 +99,11 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Haisis_SE</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Hoffer_pACD</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Haigis_SE</t>
   </si>
 </sst>
 </file>
@@ -560,7 +559,7 @@
         <v>15</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>9</v>
@@ -578,7 +577,7 @@
         <v>16</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>